<commit_message>
fix: bugs.md findings — PID race, freeze contradiction, data duplicates
- P1: PID file written AFTER bind, only unlinked if still our PID
- P2: MLB nested parameter_freezes_allowed: false → true
- P2: Deduplicated mlb_games_all.jsonl (14 dupes, 7817→7803)
- 322 tests pass, ruff clean
</commit_message>
<xml_diff>
--- a/data/research.xlsx
+++ b/data/research.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CM77" headerRowCount="1">
-  <autoFilter ref="A1:CM77"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CM79" headerRowCount="1">
+  <autoFilter ref="A1:CM79"/>
   <tableColumns count="91">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -750,19 +750,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$77)</f>
+        <f>COUNTA('Picks'!$A$2:$A$79)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$77,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$79,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$77,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$79,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$77,"settled",'Picks'!$V$2:$V$77,"win")+COUNTIFS('Picks'!$U$2:$U$77,"settled",'Picks'!$V$2:$V$77,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"win")+COUNTIFS('Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -790,19 +790,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$77,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$79,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$77,"&gt;0",'Picks'!$V$2:$V$77,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$77,"&gt;0",'Picks'!$V$2:$V$77,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$79,"&gt;0",'Picks'!$V$2:$V$79,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$79,"&gt;0",'Picks'!$V$2:$V$79,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$77,"&gt;0",'Picks'!$V$2:$V$77,"win")/(COUNTIFS('Picks'!$BX$2:$BX$77,"&gt;0",'Picks'!$V$2:$V$77,"win")+COUNTIFS('Picks'!$BX$2:$BX$77,"&gt;0",'Picks'!$V$2:$V$77,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$79,"&gt;0",'Picks'!$V$2:$V$79,"win")/(COUNTIFS('Picks'!$BX$2:$BX$79,"&gt;0",'Picks'!$V$2:$V$79,"win")+COUNTIFS('Picks'!$BX$2:$BX$79,"&gt;0",'Picks'!$V$2:$V$79,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$77)/SUM('Picks'!$BX$2:$BX$77),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$79)/SUM('Picks'!$BX$2:$BX$79),0)</f>
         <v/>
       </c>
     </row>
@@ -830,19 +830,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$77)</f>
+        <f>SUM('Picks'!$BY$2:$BY$79)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$77,"&lt;&gt;",'Picks'!$AB$2:$AB$77),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$79,"&lt;&gt;",'Picks'!$AB$2:$AB$79),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$77,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$77,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$79,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$79,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$77,'Picks'!$AM$2:$AM$77,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$79,'Picks'!$AM$2:$AM$79,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -897,15 +897,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$77,$A14,'Picks'!$U$2:$U$77,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$79,$A14,'Picks'!$U$2:$U$79,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$77,$A14,'Picks'!$U$2:$U$77,"settled",'Picks'!$V$2:$V$77,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$79,$A14,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$77,$A14,'Picks'!$U$2:$U$77,"settled",'Picks'!$V$2:$V$77,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$79,$A14,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -913,11 +913,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$77,'Picks'!$H$2:$H$77,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$79,'Picks'!$H$2:$H$79,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$77,'Picks'!$H$2:$H$77,$A14,'Picks'!$U$2:$U$77,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$79,'Picks'!$H$2:$H$79,$A14,'Picks'!$U$2:$U$79,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -928,15 +928,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$77,$A15,'Picks'!$U$2:$U$77,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$79,$A15,'Picks'!$U$2:$U$79,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$77,$A15,'Picks'!$U$2:$U$77,"settled",'Picks'!$V$2:$V$77,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$79,$A15,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$77,$A15,'Picks'!$U$2:$U$77,"settled",'Picks'!$V$2:$V$77,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$79,$A15,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -944,11 +944,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$77,'Picks'!$H$2:$H$77,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$79,'Picks'!$H$2:$H$79,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$77,'Picks'!$H$2:$H$77,$A15,'Picks'!$U$2:$U$77,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$79,'Picks'!$H$2:$H$79,$A15,'Picks'!$U$2:$U$79,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -959,15 +959,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$77,$A16,'Picks'!$U$2:$U$77,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$79,$A16,'Picks'!$U$2:$U$79,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$77,$A16,'Picks'!$U$2:$U$77,"settled",'Picks'!$V$2:$V$77,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$79,$A16,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$77,$A16,'Picks'!$U$2:$U$77,"settled",'Picks'!$V$2:$V$77,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$79,$A16,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -975,11 +975,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$77,'Picks'!$H$2:$H$77,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$79,'Picks'!$H$2:$H$79,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$77,'Picks'!$H$2:$H$77,$A16,'Picks'!$U$2:$U$77,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$79,'Picks'!$H$2:$H$79,$A16,'Picks'!$U$2:$U$79,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CM77"/>
+  <dimension ref="A1:CM79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21615,6 +21615,524 @@
       <c r="CL77" s="24" t="n"/>
       <c r="CM77" s="24" t="n"/>
     </row>
+    <row r="78" ht="36" customHeight="1">
+      <c r="A78" s="24" t="inlineStr">
+        <is>
+          <t>6bcb59f85a5f4db0</t>
+        </is>
+      </c>
+      <c r="B78" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:26:25.160034Z</t>
+        </is>
+      </c>
+      <c r="C78" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T21:00:00Z</t>
+        </is>
+      </c>
+      <c r="D78" s="24" t="inlineStr">
+        <is>
+          <t>58238</t>
+        </is>
+      </c>
+      <c r="E78" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F78" s="24" t="inlineStr">
+        <is>
+          <t>White Dragons</t>
+        </is>
+      </c>
+      <c r="G78" s="24" t="inlineStr">
+        <is>
+          <t>Role Swappers</t>
+        </is>
+      </c>
+      <c r="H78" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I78" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J78" s="25" t="n"/>
+      <c r="K78" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L78" s="26" t="n">
+        <v>186</v>
+      </c>
+      <c r="M78" s="27" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="N78" s="28" t="n">
+        <v>0.34965</v>
+      </c>
+      <c r="O78" s="28" t="n">
+        <v>0.513854</v>
+      </c>
+      <c r="P78" s="28" t="n"/>
+      <c r="Q78" s="28" t="n">
+        <v>0.164204</v>
+      </c>
+      <c r="R78" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S78" s="29" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="T78" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U78" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V78" s="24" t="n"/>
+      <c r="W78" s="26" t="n"/>
+      <c r="X78" s="26" t="n"/>
+      <c r="Y78" s="25" t="n"/>
+      <c r="Z78" s="26" t="n"/>
+      <c r="AA78" s="28" t="n"/>
+      <c r="AB78" s="28" t="n"/>
+      <c r="AC78" s="30" t="n"/>
+      <c r="AD78" s="24" t="n"/>
+      <c r="AE78" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.3500 (market_slug=aec-lol-role-wd-2026-07-23).</t>
+        </is>
+      </c>
+      <c r="AF78" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG78" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH78" s="24" t="n"/>
+      <c r="AI78" s="31" t="n"/>
+      <c r="AJ78" s="31" t="n"/>
+      <c r="AK78" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL78" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM78" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN78" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO78" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP78" s="24" t="inlineStr">
+        <is>
+          <t>White Dragons</t>
+        </is>
+      </c>
+      <c r="AQ78" s="24" t="inlineStr">
+        <is>
+          <t>White Dragons</t>
+        </is>
+      </c>
+      <c r="AR78" s="24" t="inlineStr">
+        <is>
+          <t>White Dragons</t>
+        </is>
+      </c>
+      <c r="AS78" s="24" t="inlineStr">
+        <is>
+          <t>Role Swappers</t>
+        </is>
+      </c>
+      <c r="AT78" s="24" t="inlineStr">
+        <is>
+          <t>Role Swappers</t>
+        </is>
+      </c>
+      <c r="AU78" s="24" t="inlineStr">
+        <is>
+          <t>Role Swappers</t>
+        </is>
+      </c>
+      <c r="AV78" s="24" t="n"/>
+      <c r="AW78" s="24" t="n"/>
+      <c r="AX78" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY78" s="24" t="n"/>
+      <c r="AZ78" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA78" s="24" t="inlineStr">
+        <is>
+          <t>dbc38ecdb090b63690db810d40eb29d0a69435c83dfbf24eb00d22aa42c177ae</t>
+        </is>
+      </c>
+      <c r="BB78" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC78" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD78" s="24" t="inlineStr">
+        <is>
+          <t>dbc38ecdb090b63690db810d40eb29d0a69435c83dfbf24eb00d22aa42c177ae</t>
+        </is>
+      </c>
+      <c r="BE78" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF78" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG78" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH78" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:26:14.981806Z</t>
+        </is>
+      </c>
+      <c r="BI78" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ78" s="25" t="n"/>
+      <c r="BK78" s="26" t="n">
+        <v>186</v>
+      </c>
+      <c r="BL78" s="27" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="BM78" s="28" t="n">
+        <v>0.34965</v>
+      </c>
+      <c r="BN78" s="28" t="n"/>
+      <c r="BO78" s="28" t="n"/>
+      <c r="BP78" s="25" t="n"/>
+      <c r="BQ78" s="27" t="n"/>
+      <c r="BR78" s="28" t="n"/>
+      <c r="BS78" s="28" t="n"/>
+      <c r="BT78" s="28" t="n"/>
+      <c r="BU78" s="25" t="n"/>
+      <c r="BV78" s="29" t="n"/>
+      <c r="BW78" s="24" t="n"/>
+      <c r="BX78" s="30" t="n"/>
+      <c r="BY78" s="27" t="n"/>
+      <c r="BZ78" s="24" t="n"/>
+      <c r="CA78" s="31" t="n"/>
+      <c r="CB78" s="24" t="n"/>
+      <c r="CC78" s="24" t="n"/>
+      <c r="CD78" s="24" t="n"/>
+      <c r="CE78" s="24" t="n"/>
+      <c r="CF78" s="24" t="n"/>
+      <c r="CG78" s="24" t="n"/>
+      <c r="CH78" s="24" t="n"/>
+      <c r="CI78" s="24" t="n"/>
+      <c r="CJ78" s="24" t="n"/>
+      <c r="CK78" s="24" t="n"/>
+      <c r="CL78" s="24" t="n"/>
+      <c r="CM78" s="24" t="n"/>
+    </row>
+    <row r="79" ht="36" customHeight="1">
+      <c r="A79" s="24" t="inlineStr">
+        <is>
+          <t>90b3d877e20d4290</t>
+        </is>
+      </c>
+      <c r="B79" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:27:00.632921Z</t>
+        </is>
+      </c>
+      <c r="C79" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T18:30:00Z</t>
+        </is>
+      </c>
+      <c r="D79" s="24" t="inlineStr">
+        <is>
+          <t>59850</t>
+        </is>
+      </c>
+      <c r="E79" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F79" s="24" t="inlineStr">
+        <is>
+          <t>NEW VISION</t>
+        </is>
+      </c>
+      <c r="G79" s="24" t="inlineStr">
+        <is>
+          <t>ENRAGE</t>
+        </is>
+      </c>
+      <c r="H79" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I79" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J79" s="25" t="n"/>
+      <c r="K79" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L79" s="26" t="n">
+        <v>113</v>
+      </c>
+      <c r="M79" s="27" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="N79" s="28" t="n">
+        <v>0.469484</v>
+      </c>
+      <c r="O79" s="28" t="n">
+        <v>0.504359</v>
+      </c>
+      <c r="P79" s="28" t="n"/>
+      <c r="Q79" s="28" t="n">
+        <v>0.034875</v>
+      </c>
+      <c r="R79" s="26" t="n">
+        <v>37</v>
+      </c>
+      <c r="S79" s="29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T79" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U79" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V79" s="24" t="n"/>
+      <c r="W79" s="26" t="n"/>
+      <c r="X79" s="26" t="n"/>
+      <c r="Y79" s="25" t="n"/>
+      <c r="Z79" s="26" t="n"/>
+      <c r="AA79" s="28" t="n"/>
+      <c r="AB79" s="28" t="n"/>
+      <c r="AC79" s="30" t="n"/>
+      <c r="AD79" s="24" t="n"/>
+      <c r="AE79" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.4700 (market_slug=aec-cs2-enr-nve-2026-07-23).</t>
+        </is>
+      </c>
+      <c r="AF79" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG79" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH79" s="24" t="n"/>
+      <c r="AI79" s="31" t="n"/>
+      <c r="AJ79" s="31" t="n"/>
+      <c r="AK79" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL79" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM79" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN79" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO79" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP79" s="24" t="inlineStr">
+        <is>
+          <t>NEW VISION</t>
+        </is>
+      </c>
+      <c r="AQ79" s="24" t="inlineStr">
+        <is>
+          <t>NEW VISION</t>
+        </is>
+      </c>
+      <c r="AR79" s="24" t="inlineStr">
+        <is>
+          <t>NEW VISION</t>
+        </is>
+      </c>
+      <c r="AS79" s="24" t="inlineStr">
+        <is>
+          <t>ENRAGE</t>
+        </is>
+      </c>
+      <c r="AT79" s="24" t="inlineStr">
+        <is>
+          <t>ENRAGE</t>
+        </is>
+      </c>
+      <c r="AU79" s="24" t="inlineStr">
+        <is>
+          <t>ENRAGE</t>
+        </is>
+      </c>
+      <c r="AV79" s="24" t="n"/>
+      <c r="AW79" s="24" t="n"/>
+      <c r="AX79" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY79" s="24" t="n"/>
+      <c r="AZ79" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA79" s="24" t="inlineStr">
+        <is>
+          <t>48424b79d75fc1173c9c465d95feb6fc041a2ccfbc64455058b3f74905ce28d5</t>
+        </is>
+      </c>
+      <c r="BB79" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC79" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD79" s="24" t="inlineStr">
+        <is>
+          <t>48424b79d75fc1173c9c465d95feb6fc041a2ccfbc64455058b3f74905ce28d5</t>
+        </is>
+      </c>
+      <c r="BE79" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF79" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG79" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH79" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:26:40.388327Z</t>
+        </is>
+      </c>
+      <c r="BI79" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ79" s="25" t="n"/>
+      <c r="BK79" s="26" t="n">
+        <v>113</v>
+      </c>
+      <c r="BL79" s="27" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="BM79" s="28" t="n">
+        <v>0.469484</v>
+      </c>
+      <c r="BN79" s="28" t="n"/>
+      <c r="BO79" s="28" t="n"/>
+      <c r="BP79" s="25" t="n"/>
+      <c r="BQ79" s="27" t="n"/>
+      <c r="BR79" s="28" t="n"/>
+      <c r="BS79" s="28" t="n"/>
+      <c r="BT79" s="28" t="n"/>
+      <c r="BU79" s="25" t="n"/>
+      <c r="BV79" s="29" t="n"/>
+      <c r="BW79" s="24" t="n"/>
+      <c r="BX79" s="30" t="n"/>
+      <c r="BY79" s="27" t="n"/>
+      <c r="BZ79" s="24" t="n"/>
+      <c r="CA79" s="31" t="n"/>
+      <c r="CB79" s="24" t="n"/>
+      <c r="CC79" s="24" t="n"/>
+      <c r="CD79" s="24" t="n"/>
+      <c r="CE79" s="24" t="n"/>
+      <c r="CF79" s="24" t="n"/>
+      <c r="CG79" s="24" t="n"/>
+      <c r="CH79" s="24" t="n"/>
+      <c r="CI79" s="24" t="n"/>
+      <c r="CJ79" s="24" t="n"/>
+      <c r="CK79" s="24" t="n"/>
+      <c r="CL79" s="24" t="n"/>
+      <c r="CM79" s="24" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
all: remaining runtime + code changes
</commit_message>
<xml_diff>
--- a/data/research.xlsx
+++ b/data/research.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CM79" headerRowCount="1">
-  <autoFilter ref="A1:CM79"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CM85" headerRowCount="1">
+  <autoFilter ref="A1:CM85"/>
   <tableColumns count="91">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -750,19 +750,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$79)</f>
+        <f>COUNTA('Picks'!$A$2:$A$85)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$79,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$85,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$79,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$85,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"win")+COUNTIFS('Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$85,"settled",'Picks'!$V$2:$V$85,"win")+COUNTIFS('Picks'!$U$2:$U$85,"settled",'Picks'!$V$2:$V$85,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -790,19 +790,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$79,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$85,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$79,"&gt;0",'Picks'!$V$2:$V$79,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$79,"&gt;0",'Picks'!$V$2:$V$79,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$85,"&gt;0",'Picks'!$V$2:$V$85,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$85,"&gt;0",'Picks'!$V$2:$V$85,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$79,"&gt;0",'Picks'!$V$2:$V$79,"win")/(COUNTIFS('Picks'!$BX$2:$BX$79,"&gt;0",'Picks'!$V$2:$V$79,"win")+COUNTIFS('Picks'!$BX$2:$BX$79,"&gt;0",'Picks'!$V$2:$V$79,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$85,"&gt;0",'Picks'!$V$2:$V$85,"win")/(COUNTIFS('Picks'!$BX$2:$BX$85,"&gt;0",'Picks'!$V$2:$V$85,"win")+COUNTIFS('Picks'!$BX$2:$BX$85,"&gt;0",'Picks'!$V$2:$V$85,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$79)/SUM('Picks'!$BX$2:$BX$79),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$85)/SUM('Picks'!$BX$2:$BX$85),0)</f>
         <v/>
       </c>
     </row>
@@ -830,19 +830,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$79)</f>
+        <f>SUM('Picks'!$BY$2:$BY$85)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$79,"&lt;&gt;",'Picks'!$AB$2:$AB$79),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$85,"&lt;&gt;",'Picks'!$AB$2:$AB$85),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$79,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$79,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$85,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$85,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$79,'Picks'!$AM$2:$AM$79,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$85,'Picks'!$AM$2:$AM$85,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -897,15 +897,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$79,$A14,'Picks'!$U$2:$U$79,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$85,$A14,'Picks'!$U$2:$U$85,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$79,$A14,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$85,$A14,'Picks'!$U$2:$U$85,"settled",'Picks'!$V$2:$V$85,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$79,$A14,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$85,$A14,'Picks'!$U$2:$U$85,"settled",'Picks'!$V$2:$V$85,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -913,11 +913,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$79,'Picks'!$H$2:$H$79,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$85,'Picks'!$H$2:$H$85,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$79,'Picks'!$H$2:$H$79,$A14,'Picks'!$U$2:$U$79,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$85,'Picks'!$H$2:$H$85,$A14,'Picks'!$U$2:$U$85,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -928,15 +928,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$79,$A15,'Picks'!$U$2:$U$79,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$85,$A15,'Picks'!$U$2:$U$85,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$79,$A15,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$85,$A15,'Picks'!$U$2:$U$85,"settled",'Picks'!$V$2:$V$85,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$79,$A15,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$85,$A15,'Picks'!$U$2:$U$85,"settled",'Picks'!$V$2:$V$85,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -944,11 +944,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$79,'Picks'!$H$2:$H$79,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$85,'Picks'!$H$2:$H$85,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$79,'Picks'!$H$2:$H$79,$A15,'Picks'!$U$2:$U$79,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$85,'Picks'!$H$2:$H$85,$A15,'Picks'!$U$2:$U$85,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -959,15 +959,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$79,$A16,'Picks'!$U$2:$U$79,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$85,$A16,'Picks'!$U$2:$U$85,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$79,$A16,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$85,$A16,'Picks'!$U$2:$U$85,"settled",'Picks'!$V$2:$V$85,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$79,$A16,'Picks'!$U$2:$U$79,"settled",'Picks'!$V$2:$V$79,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$85,$A16,'Picks'!$U$2:$U$85,"settled",'Picks'!$V$2:$V$85,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -975,11 +975,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$79,'Picks'!$H$2:$H$79,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$85,'Picks'!$H$2:$H$85,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$79,'Picks'!$H$2:$H$79,$A16,'Picks'!$U$2:$U$79,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$85,'Picks'!$H$2:$H$85,$A16,'Picks'!$U$2:$U$85,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CM79"/>
+  <dimension ref="A1:CM85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3527,18 +3527,32 @@
       </c>
       <c r="U9" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V9" s="24" t="n"/>
-      <c r="W9" s="26" t="n"/>
-      <c r="X9" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V9" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W9" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X9" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="Y9" s="25" t="n"/>
       <c r="Z9" s="26" t="n"/>
       <c r="AA9" s="28" t="n"/>
       <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="30" t="n"/>
-      <c r="AD9" s="24" t="n"/>
+      <c r="AC9" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:34:29.539199Z</t>
+        </is>
+      </c>
       <c r="AE9" s="31" t="inlineStr">
         <is>
           <t>Neutral Elo baseline; executable ask 0.4000 (market_slug=aec-cs2-100t-ntr-2026-07-23).</t>
@@ -12788,18 +12802,32 @@
       </c>
       <c r="U44" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V44" s="24" t="n"/>
-      <c r="W44" s="26" t="n"/>
-      <c r="X44" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V44" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W44" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X44" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="Y44" s="25" t="n"/>
       <c r="Z44" s="26" t="n"/>
       <c r="AA44" s="28" t="n"/>
       <c r="AB44" s="28" t="n"/>
-      <c r="AC44" s="30" t="n"/>
-      <c r="AD44" s="24" t="n"/>
+      <c r="AC44" s="30" t="n">
+        <v>1.875</v>
+      </c>
+      <c r="AD44" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:34:40.105334Z</t>
+        </is>
+      </c>
       <c r="AE44" s="31" t="inlineStr">
         <is>
           <t>Neutral Elo baseline; executable ask 0.4000 (market_slug=aec-cs2-100t-ntr-2026-07-23).</t>
@@ -22133,6 +22161,1560 @@
       <c r="CL79" s="24" t="n"/>
       <c r="CM79" s="24" t="n"/>
     </row>
+    <row r="80" ht="36" customHeight="1">
+      <c r="A80" s="24" t="inlineStr">
+        <is>
+          <t>2d3f5fba93944fa5</t>
+        </is>
+      </c>
+      <c r="B80" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:35:50.881798Z</t>
+        </is>
+      </c>
+      <c r="C80" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="D80" s="24" t="inlineStr">
+        <is>
+          <t>58235</t>
+        </is>
+      </c>
+      <c r="E80" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F80" s="24" t="inlineStr">
+        <is>
+          <t>EXSAD Gaming</t>
+        </is>
+      </c>
+      <c r="G80" s="24" t="inlineStr">
+        <is>
+          <t>Capybara Esports</t>
+        </is>
+      </c>
+      <c r="H80" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I80" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J80" s="25" t="n"/>
+      <c r="K80" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L80" s="26" t="n">
+        <v>-186</v>
+      </c>
+      <c r="M80" s="27" t="n">
+        <v>1.537634</v>
+      </c>
+      <c r="N80" s="28" t="n">
+        <v>0.65035</v>
+      </c>
+      <c r="O80" s="28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P80" s="28" t="n"/>
+      <c r="Q80" s="28" t="n">
+        <v>-0.15035</v>
+      </c>
+      <c r="R80" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S80" s="29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T80" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U80" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V80" s="24" t="n"/>
+      <c r="W80" s="26" t="n"/>
+      <c r="X80" s="26" t="n"/>
+      <c r="Y80" s="25" t="n"/>
+      <c r="Z80" s="26" t="n"/>
+      <c r="AA80" s="28" t="n"/>
+      <c r="AB80" s="28" t="n"/>
+      <c r="AC80" s="30" t="n"/>
+      <c r="AD80" s="24" t="n"/>
+      <c r="AE80" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6500 (market_slug=aec-lol-capy-exg-2026-07-23).</t>
+        </is>
+      </c>
+      <c r="AF80" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG80" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH80" s="24" t="n"/>
+      <c r="AI80" s="31" t="n"/>
+      <c r="AJ80" s="31" t="n"/>
+      <c r="AK80" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL80" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM80" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN80" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO80" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP80" s="24" t="inlineStr">
+        <is>
+          <t>EXSAD Gaming</t>
+        </is>
+      </c>
+      <c r="AQ80" s="24" t="inlineStr">
+        <is>
+          <t>EXSAD Gaming</t>
+        </is>
+      </c>
+      <c r="AR80" s="24" t="inlineStr">
+        <is>
+          <t>EXSAD Gaming</t>
+        </is>
+      </c>
+      <c r="AS80" s="24" t="inlineStr">
+        <is>
+          <t>Capybara Esports</t>
+        </is>
+      </c>
+      <c r="AT80" s="24" t="inlineStr">
+        <is>
+          <t>Capybara Esports</t>
+        </is>
+      </c>
+      <c r="AU80" s="24" t="inlineStr">
+        <is>
+          <t>Capybara Esports</t>
+        </is>
+      </c>
+      <c r="AV80" s="24" t="n"/>
+      <c r="AW80" s="24" t="n"/>
+      <c r="AX80" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY80" s="24" t="n"/>
+      <c r="AZ80" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA80" s="24" t="inlineStr">
+        <is>
+          <t>dbc38ecdb090b63690db810d40eb29d0a69435c83dfbf24eb00d22aa42c177ae</t>
+        </is>
+      </c>
+      <c r="BB80" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC80" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD80" s="24" t="inlineStr">
+        <is>
+          <t>dbc38ecdb090b63690db810d40eb29d0a69435c83dfbf24eb00d22aa42c177ae</t>
+        </is>
+      </c>
+      <c r="BE80" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF80" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG80" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH80" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:35:35.265338Z</t>
+        </is>
+      </c>
+      <c r="BI80" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ80" s="25" t="n"/>
+      <c r="BK80" s="26" t="n">
+        <v>-186</v>
+      </c>
+      <c r="BL80" s="27" t="n">
+        <v>1.537634</v>
+      </c>
+      <c r="BM80" s="28" t="n">
+        <v>0.65035</v>
+      </c>
+      <c r="BN80" s="28" t="n"/>
+      <c r="BO80" s="28" t="n"/>
+      <c r="BP80" s="25" t="n"/>
+      <c r="BQ80" s="27" t="n"/>
+      <c r="BR80" s="28" t="n"/>
+      <c r="BS80" s="28" t="n"/>
+      <c r="BT80" s="28" t="n"/>
+      <c r="BU80" s="25" t="n"/>
+      <c r="BV80" s="29" t="n"/>
+      <c r="BW80" s="24" t="n"/>
+      <c r="BX80" s="30" t="n"/>
+      <c r="BY80" s="27" t="n"/>
+      <c r="BZ80" s="24" t="n"/>
+      <c r="CA80" s="31" t="n"/>
+      <c r="CB80" s="24" t="n"/>
+      <c r="CC80" s="24" t="n"/>
+      <c r="CD80" s="24" t="n"/>
+      <c r="CE80" s="24" t="n"/>
+      <c r="CF80" s="24" t="n"/>
+      <c r="CG80" s="24" t="n"/>
+      <c r="CH80" s="24" t="n"/>
+      <c r="CI80" s="24" t="n"/>
+      <c r="CJ80" s="24" t="n"/>
+      <c r="CK80" s="24" t="n"/>
+      <c r="CL80" s="24" t="n"/>
+      <c r="CM80" s="24" t="n"/>
+    </row>
+    <row r="81" ht="36" customHeight="1">
+      <c r="A81" s="24" t="inlineStr">
+        <is>
+          <t>fbfa8685a306416e</t>
+        </is>
+      </c>
+      <c r="B81" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:35:50.881798Z</t>
+        </is>
+      </c>
+      <c r="C81" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-24T16:00:00Z</t>
+        </is>
+      </c>
+      <c r="D81" s="24" t="inlineStr">
+        <is>
+          <t>58454</t>
+        </is>
+      </c>
+      <c r="E81" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F81" s="24" t="inlineStr">
+        <is>
+          <t>GMBLERS ESPORTS</t>
+        </is>
+      </c>
+      <c r="G81" s="24" t="inlineStr">
+        <is>
+          <t>P11 Esports</t>
+        </is>
+      </c>
+      <c r="H81" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I81" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J81" s="25" t="n"/>
+      <c r="K81" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L81" s="26" t="n">
+        <v>133</v>
+      </c>
+      <c r="M81" s="27" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="N81" s="28" t="n">
+        <v>0.429185</v>
+      </c>
+      <c r="O81" s="28" t="n">
+        <v>0.5851769999999999</v>
+      </c>
+      <c r="P81" s="28" t="n"/>
+      <c r="Q81" s="28" t="n">
+        <v>0.155992</v>
+      </c>
+      <c r="R81" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S81" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T81" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U81" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V81" s="24" t="n"/>
+      <c r="W81" s="26" t="n"/>
+      <c r="X81" s="26" t="n"/>
+      <c r="Y81" s="25" t="n"/>
+      <c r="Z81" s="26" t="n"/>
+      <c r="AA81" s="28" t="n"/>
+      <c r="AB81" s="28" t="n"/>
+      <c r="AC81" s="30" t="n"/>
+      <c r="AD81" s="24" t="n"/>
+      <c r="AE81" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.4300 (market_slug=aec-lol-p11-gmb-2026-07-24).</t>
+        </is>
+      </c>
+      <c r="AF81" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG81" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH81" s="24" t="n"/>
+      <c r="AI81" s="31" t="n"/>
+      <c r="AJ81" s="31" t="n"/>
+      <c r="AK81" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL81" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM81" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN81" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO81" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP81" s="24" t="inlineStr">
+        <is>
+          <t>GMBLERS ESPORTS</t>
+        </is>
+      </c>
+      <c r="AQ81" s="24" t="inlineStr">
+        <is>
+          <t>GMBLERS ESPORTS</t>
+        </is>
+      </c>
+      <c r="AR81" s="24" t="inlineStr">
+        <is>
+          <t>GMBLERS ESPORTS</t>
+        </is>
+      </c>
+      <c r="AS81" s="24" t="inlineStr">
+        <is>
+          <t>P11 Esports</t>
+        </is>
+      </c>
+      <c r="AT81" s="24" t="inlineStr">
+        <is>
+          <t>P11 Esports</t>
+        </is>
+      </c>
+      <c r="AU81" s="24" t="inlineStr">
+        <is>
+          <t>P11 Esports</t>
+        </is>
+      </c>
+      <c r="AV81" s="24" t="n"/>
+      <c r="AW81" s="24" t="n"/>
+      <c r="AX81" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY81" s="24" t="n"/>
+      <c r="AZ81" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA81" s="24" t="inlineStr">
+        <is>
+          <t>dbc38ecdb090b63690db810d40eb29d0a69435c83dfbf24eb00d22aa42c177ae</t>
+        </is>
+      </c>
+      <c r="BB81" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC81" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD81" s="24" t="inlineStr">
+        <is>
+          <t>dbc38ecdb090b63690db810d40eb29d0a69435c83dfbf24eb00d22aa42c177ae</t>
+        </is>
+      </c>
+      <c r="BE81" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF81" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG81" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH81" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:35:47.586016Z</t>
+        </is>
+      </c>
+      <c r="BI81" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ81" s="25" t="n"/>
+      <c r="BK81" s="26" t="n">
+        <v>133</v>
+      </c>
+      <c r="BL81" s="27" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="BM81" s="28" t="n">
+        <v>0.429185</v>
+      </c>
+      <c r="BN81" s="28" t="n"/>
+      <c r="BO81" s="28" t="n"/>
+      <c r="BP81" s="25" t="n"/>
+      <c r="BQ81" s="27" t="n"/>
+      <c r="BR81" s="28" t="n"/>
+      <c r="BS81" s="28" t="n"/>
+      <c r="BT81" s="28" t="n"/>
+      <c r="BU81" s="25" t="n"/>
+      <c r="BV81" s="29" t="n"/>
+      <c r="BW81" s="24" t="n"/>
+      <c r="BX81" s="30" t="n"/>
+      <c r="BY81" s="27" t="n"/>
+      <c r="BZ81" s="24" t="n"/>
+      <c r="CA81" s="31" t="n"/>
+      <c r="CB81" s="24" t="n"/>
+      <c r="CC81" s="24" t="n"/>
+      <c r="CD81" s="24" t="n"/>
+      <c r="CE81" s="24" t="n"/>
+      <c r="CF81" s="24" t="n"/>
+      <c r="CG81" s="24" t="n"/>
+      <c r="CH81" s="24" t="n"/>
+      <c r="CI81" s="24" t="n"/>
+      <c r="CJ81" s="24" t="n"/>
+      <c r="CK81" s="24" t="n"/>
+      <c r="CL81" s="24" t="n"/>
+      <c r="CM81" s="24" t="n"/>
+    </row>
+    <row r="82" ht="36" customHeight="1">
+      <c r="A82" s="24" t="inlineStr">
+        <is>
+          <t>b948ea8c0be54c58</t>
+        </is>
+      </c>
+      <c r="B82" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:36:27.605488Z</t>
+        </is>
+      </c>
+      <c r="C82" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-24T16:00:00Z</t>
+        </is>
+      </c>
+      <c r="D82" s="24" t="inlineStr">
+        <is>
+          <t>60130</t>
+        </is>
+      </c>
+      <c r="E82" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F82" s="24" t="inlineStr">
+        <is>
+          <t>Walczaki</t>
+        </is>
+      </c>
+      <c r="G82" s="24" t="inlineStr">
+        <is>
+          <t>Gentle Mates</t>
+        </is>
+      </c>
+      <c r="H82" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I82" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J82" s="25" t="n"/>
+      <c r="K82" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L82" s="26" t="n">
+        <v>-203</v>
+      </c>
+      <c r="M82" s="27" t="n">
+        <v>1.492611</v>
+      </c>
+      <c r="N82" s="28" t="n">
+        <v>0.669967</v>
+      </c>
+      <c r="O82" s="28" t="n">
+        <v>0.517334</v>
+      </c>
+      <c r="P82" s="28" t="n"/>
+      <c r="Q82" s="28" t="n">
+        <v>-0.152633</v>
+      </c>
+      <c r="R82" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S82" s="29" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="T82" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U82" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V82" s="24" t="n"/>
+      <c r="W82" s="26" t="n"/>
+      <c r="X82" s="26" t="n"/>
+      <c r="Y82" s="25" t="n"/>
+      <c r="Z82" s="26" t="n"/>
+      <c r="AA82" s="28" t="n"/>
+      <c r="AB82" s="28" t="n"/>
+      <c r="AC82" s="30" t="n"/>
+      <c r="AD82" s="24" t="n"/>
+      <c r="AE82" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6700 (market_slug=aec-cs2-m8-wal-2026-07-24).</t>
+        </is>
+      </c>
+      <c r="AF82" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG82" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH82" s="24" t="n"/>
+      <c r="AI82" s="31" t="n"/>
+      <c r="AJ82" s="31" t="n"/>
+      <c r="AK82" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL82" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM82" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN82" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO82" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP82" s="24" t="inlineStr">
+        <is>
+          <t>Walczaki</t>
+        </is>
+      </c>
+      <c r="AQ82" s="24" t="inlineStr">
+        <is>
+          <t>Walczaki</t>
+        </is>
+      </c>
+      <c r="AR82" s="24" t="inlineStr">
+        <is>
+          <t>Walczaki</t>
+        </is>
+      </c>
+      <c r="AS82" s="24" t="inlineStr">
+        <is>
+          <t>Gentle Mates</t>
+        </is>
+      </c>
+      <c r="AT82" s="24" t="inlineStr">
+        <is>
+          <t>Gentle Mates</t>
+        </is>
+      </c>
+      <c r="AU82" s="24" t="inlineStr">
+        <is>
+          <t>Gentle Mates</t>
+        </is>
+      </c>
+      <c r="AV82" s="24" t="n"/>
+      <c r="AW82" s="24" t="n"/>
+      <c r="AX82" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY82" s="24" t="n"/>
+      <c r="AZ82" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA82" s="24" t="inlineStr">
+        <is>
+          <t>48424b79d75fc1173c9c465d95feb6fc041a2ccfbc64455058b3f74905ce28d5</t>
+        </is>
+      </c>
+      <c r="BB82" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC82" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD82" s="24" t="inlineStr">
+        <is>
+          <t>48424b79d75fc1173c9c465d95feb6fc041a2ccfbc64455058b3f74905ce28d5</t>
+        </is>
+      </c>
+      <c r="BE82" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF82" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG82" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH82" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:36:22.454543Z</t>
+        </is>
+      </c>
+      <c r="BI82" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ82" s="25" t="n"/>
+      <c r="BK82" s="26" t="n">
+        <v>-203</v>
+      </c>
+      <c r="BL82" s="27" t="n">
+        <v>1.492611</v>
+      </c>
+      <c r="BM82" s="28" t="n">
+        <v>0.669967</v>
+      </c>
+      <c r="BN82" s="28" t="n"/>
+      <c r="BO82" s="28" t="n"/>
+      <c r="BP82" s="25" t="n"/>
+      <c r="BQ82" s="27" t="n"/>
+      <c r="BR82" s="28" t="n"/>
+      <c r="BS82" s="28" t="n"/>
+      <c r="BT82" s="28" t="n"/>
+      <c r="BU82" s="25" t="n"/>
+      <c r="BV82" s="29" t="n"/>
+      <c r="BW82" s="24" t="n"/>
+      <c r="BX82" s="30" t="n"/>
+      <c r="BY82" s="27" t="n"/>
+      <c r="BZ82" s="24" t="n"/>
+      <c r="CA82" s="31" t="n"/>
+      <c r="CB82" s="24" t="n"/>
+      <c r="CC82" s="24" t="n"/>
+      <c r="CD82" s="24" t="n"/>
+      <c r="CE82" s="24" t="n"/>
+      <c r="CF82" s="24" t="n"/>
+      <c r="CG82" s="24" t="n"/>
+      <c r="CH82" s="24" t="n"/>
+      <c r="CI82" s="24" t="n"/>
+      <c r="CJ82" s="24" t="n"/>
+      <c r="CK82" s="24" t="n"/>
+      <c r="CL82" s="24" t="n"/>
+      <c r="CM82" s="24" t="n"/>
+    </row>
+    <row r="83" ht="36" customHeight="1">
+      <c r="A83" s="24" t="inlineStr">
+        <is>
+          <t>ec5f8d7b7b024e96</t>
+        </is>
+      </c>
+      <c r="B83" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:36:27.605488Z</t>
+        </is>
+      </c>
+      <c r="C83" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-24T17:00:00Z</t>
+        </is>
+      </c>
+      <c r="D83" s="24" t="inlineStr">
+        <is>
+          <t>59043</t>
+        </is>
+      </c>
+      <c r="E83" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F83" s="24" t="inlineStr">
+        <is>
+          <t>Atreides</t>
+        </is>
+      </c>
+      <c r="G83" s="24" t="inlineStr">
+        <is>
+          <t>GenOne</t>
+        </is>
+      </c>
+      <c r="H83" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I83" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J83" s="25" t="n"/>
+      <c r="K83" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L83" s="26" t="n">
+        <v>-203</v>
+      </c>
+      <c r="M83" s="27" t="n">
+        <v>1.492611</v>
+      </c>
+      <c r="N83" s="28" t="n">
+        <v>0.669967</v>
+      </c>
+      <c r="O83" s="28" t="n">
+        <v>0.5724050000000001</v>
+      </c>
+      <c r="P83" s="28" t="n"/>
+      <c r="Q83" s="28" t="n">
+        <v>-0.097562</v>
+      </c>
+      <c r="R83" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S83" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T83" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U83" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V83" s="24" t="n"/>
+      <c r="W83" s="26" t="n"/>
+      <c r="X83" s="26" t="n"/>
+      <c r="Y83" s="25" t="n"/>
+      <c r="Z83" s="26" t="n"/>
+      <c r="AA83" s="28" t="n"/>
+      <c r="AB83" s="28" t="n"/>
+      <c r="AC83" s="30" t="n"/>
+      <c r="AD83" s="24" t="n"/>
+      <c r="AE83" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6700 (market_slug=aec-cs2-g1-atr-2026-07-24).</t>
+        </is>
+      </c>
+      <c r="AF83" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG83" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH83" s="24" t="n"/>
+      <c r="AI83" s="31" t="n"/>
+      <c r="AJ83" s="31" t="n"/>
+      <c r="AK83" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL83" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM83" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN83" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO83" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP83" s="24" t="inlineStr">
+        <is>
+          <t>Atreides</t>
+        </is>
+      </c>
+      <c r="AQ83" s="24" t="inlineStr">
+        <is>
+          <t>Atreides</t>
+        </is>
+      </c>
+      <c r="AR83" s="24" t="inlineStr">
+        <is>
+          <t>Atreides</t>
+        </is>
+      </c>
+      <c r="AS83" s="24" t="inlineStr">
+        <is>
+          <t>GenOne</t>
+        </is>
+      </c>
+      <c r="AT83" s="24" t="inlineStr">
+        <is>
+          <t>GenOne</t>
+        </is>
+      </c>
+      <c r="AU83" s="24" t="inlineStr">
+        <is>
+          <t>GenOne</t>
+        </is>
+      </c>
+      <c r="AV83" s="24" t="n"/>
+      <c r="AW83" s="24" t="n"/>
+      <c r="AX83" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY83" s="24" t="n"/>
+      <c r="AZ83" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA83" s="24" t="inlineStr">
+        <is>
+          <t>48424b79d75fc1173c9c465d95feb6fc041a2ccfbc64455058b3f74905ce28d5</t>
+        </is>
+      </c>
+      <c r="BB83" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC83" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD83" s="24" t="inlineStr">
+        <is>
+          <t>48424b79d75fc1173c9c465d95feb6fc041a2ccfbc64455058b3f74905ce28d5</t>
+        </is>
+      </c>
+      <c r="BE83" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF83" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG83" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH83" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:36:23.372169Z</t>
+        </is>
+      </c>
+      <c r="BI83" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ83" s="25" t="n"/>
+      <c r="BK83" s="26" t="n">
+        <v>-203</v>
+      </c>
+      <c r="BL83" s="27" t="n">
+        <v>1.492611</v>
+      </c>
+      <c r="BM83" s="28" t="n">
+        <v>0.669967</v>
+      </c>
+      <c r="BN83" s="28" t="n"/>
+      <c r="BO83" s="28" t="n"/>
+      <c r="BP83" s="25" t="n"/>
+      <c r="BQ83" s="27" t="n"/>
+      <c r="BR83" s="28" t="n"/>
+      <c r="BS83" s="28" t="n"/>
+      <c r="BT83" s="28" t="n"/>
+      <c r="BU83" s="25" t="n"/>
+      <c r="BV83" s="29" t="n"/>
+      <c r="BW83" s="24" t="n"/>
+      <c r="BX83" s="30" t="n"/>
+      <c r="BY83" s="27" t="n"/>
+      <c r="BZ83" s="24" t="n"/>
+      <c r="CA83" s="31" t="n"/>
+      <c r="CB83" s="24" t="n"/>
+      <c r="CC83" s="24" t="n"/>
+      <c r="CD83" s="24" t="n"/>
+      <c r="CE83" s="24" t="n"/>
+      <c r="CF83" s="24" t="n"/>
+      <c r="CG83" s="24" t="n"/>
+      <c r="CH83" s="24" t="n"/>
+      <c r="CI83" s="24" t="n"/>
+      <c r="CJ83" s="24" t="n"/>
+      <c r="CK83" s="24" t="n"/>
+      <c r="CL83" s="24" t="n"/>
+      <c r="CM83" s="24" t="n"/>
+    </row>
+    <row r="84" ht="36" customHeight="1">
+      <c r="A84" s="24" t="inlineStr">
+        <is>
+          <t>0290b65f79474bcb</t>
+        </is>
+      </c>
+      <c r="B84" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:36:27.605488Z</t>
+        </is>
+      </c>
+      <c r="C84" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-24T19:00:00Z</t>
+        </is>
+      </c>
+      <c r="D84" s="24" t="inlineStr">
+        <is>
+          <t>59967</t>
+        </is>
+      </c>
+      <c r="E84" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F84" s="24" t="inlineStr">
+        <is>
+          <t>ALKA GAMING</t>
+        </is>
+      </c>
+      <c r="G84" s="24" t="inlineStr">
+        <is>
+          <t>Keyd</t>
+        </is>
+      </c>
+      <c r="H84" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I84" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J84" s="25" t="n"/>
+      <c r="K84" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L84" s="26" t="n">
+        <v>-156</v>
+      </c>
+      <c r="M84" s="27" t="n">
+        <v>1.641026</v>
+      </c>
+      <c r="N84" s="28" t="n">
+        <v>0.609375</v>
+      </c>
+      <c r="O84" s="28" t="n">
+        <v>0.568001</v>
+      </c>
+      <c r="P84" s="28" t="n"/>
+      <c r="Q84" s="28" t="n">
+        <v>-0.041374</v>
+      </c>
+      <c r="R84" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S84" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T84" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U84" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V84" s="24" t="n"/>
+      <c r="W84" s="26" t="n"/>
+      <c r="X84" s="26" t="n"/>
+      <c r="Y84" s="25" t="n"/>
+      <c r="Z84" s="26" t="n"/>
+      <c r="AA84" s="28" t="n"/>
+      <c r="AB84" s="28" t="n"/>
+      <c r="AC84" s="30" t="n"/>
+      <c r="AD84" s="24" t="n"/>
+      <c r="AE84" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6100 (market_slug=aec-cs2-keyd-alka-2026-07-24).</t>
+        </is>
+      </c>
+      <c r="AF84" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG84" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH84" s="24" t="n"/>
+      <c r="AI84" s="31" t="n"/>
+      <c r="AJ84" s="31" t="n"/>
+      <c r="AK84" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL84" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM84" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN84" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO84" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP84" s="24" t="inlineStr">
+        <is>
+          <t>ALKA GAMING</t>
+        </is>
+      </c>
+      <c r="AQ84" s="24" t="inlineStr">
+        <is>
+          <t>ALKA GAMING</t>
+        </is>
+      </c>
+      <c r="AR84" s="24" t="inlineStr">
+        <is>
+          <t>ALKA GAMING</t>
+        </is>
+      </c>
+      <c r="AS84" s="24" t="inlineStr">
+        <is>
+          <t>Keyd</t>
+        </is>
+      </c>
+      <c r="AT84" s="24" t="inlineStr">
+        <is>
+          <t>Keyd</t>
+        </is>
+      </c>
+      <c r="AU84" s="24" t="inlineStr">
+        <is>
+          <t>Keyd</t>
+        </is>
+      </c>
+      <c r="AV84" s="24" t="n"/>
+      <c r="AW84" s="24" t="n"/>
+      <c r="AX84" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY84" s="24" t="n"/>
+      <c r="AZ84" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA84" s="24" t="inlineStr">
+        <is>
+          <t>48424b79d75fc1173c9c465d95feb6fc041a2ccfbc64455058b3f74905ce28d5</t>
+        </is>
+      </c>
+      <c r="BB84" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC84" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD84" s="24" t="inlineStr">
+        <is>
+          <t>48424b79d75fc1173c9c465d95feb6fc041a2ccfbc64455058b3f74905ce28d5</t>
+        </is>
+      </c>
+      <c r="BE84" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF84" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG84" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH84" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:36:26.758550Z</t>
+        </is>
+      </c>
+      <c r="BI84" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ84" s="25" t="n"/>
+      <c r="BK84" s="26" t="n">
+        <v>-156</v>
+      </c>
+      <c r="BL84" s="27" t="n">
+        <v>1.641026</v>
+      </c>
+      <c r="BM84" s="28" t="n">
+        <v>0.609375</v>
+      </c>
+      <c r="BN84" s="28" t="n"/>
+      <c r="BO84" s="28" t="n"/>
+      <c r="BP84" s="25" t="n"/>
+      <c r="BQ84" s="27" t="n"/>
+      <c r="BR84" s="28" t="n"/>
+      <c r="BS84" s="28" t="n"/>
+      <c r="BT84" s="28" t="n"/>
+      <c r="BU84" s="25" t="n"/>
+      <c r="BV84" s="29" t="n"/>
+      <c r="BW84" s="24" t="n"/>
+      <c r="BX84" s="30" t="n"/>
+      <c r="BY84" s="27" t="n"/>
+      <c r="BZ84" s="24" t="n"/>
+      <c r="CA84" s="31" t="n"/>
+      <c r="CB84" s="24" t="n"/>
+      <c r="CC84" s="24" t="n"/>
+      <c r="CD84" s="24" t="n"/>
+      <c r="CE84" s="24" t="n"/>
+      <c r="CF84" s="24" t="n"/>
+      <c r="CG84" s="24" t="n"/>
+      <c r="CH84" s="24" t="n"/>
+      <c r="CI84" s="24" t="n"/>
+      <c r="CJ84" s="24" t="n"/>
+      <c r="CK84" s="24" t="n"/>
+      <c r="CL84" s="24" t="n"/>
+      <c r="CM84" s="24" t="n"/>
+    </row>
+    <row r="85" ht="36" customHeight="1">
+      <c r="A85" s="24" t="inlineStr">
+        <is>
+          <t>97a20129d01c4f3a</t>
+        </is>
+      </c>
+      <c r="B85" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:36:54.423225Z</t>
+        </is>
+      </c>
+      <c r="C85" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="D85" s="24" t="inlineStr">
+        <is>
+          <t>57152</t>
+        </is>
+      </c>
+      <c r="E85" s="24" t="inlineStr">
+        <is>
+          <t>VALORANT</t>
+        </is>
+      </c>
+      <c r="F85" s="24" t="inlineStr">
+        <is>
+          <t>ALTERNATE aTTaX Ruby</t>
+        </is>
+      </c>
+      <c r="G85" s="24" t="inlineStr">
+        <is>
+          <t>Karmine Corp GC</t>
+        </is>
+      </c>
+      <c r="H85" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I85" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J85" s="25" t="n"/>
+      <c r="K85" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L85" s="26" t="n">
+        <v>-163</v>
+      </c>
+      <c r="M85" s="27" t="n">
+        <v>1.613497</v>
+      </c>
+      <c r="N85" s="28" t="n">
+        <v>0.619772</v>
+      </c>
+      <c r="O85" s="28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P85" s="28" t="n"/>
+      <c r="Q85" s="28" t="n">
+        <v>-0.119772</v>
+      </c>
+      <c r="R85" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S85" s="29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T85" s="24" t="inlineStr">
+        <is>
+          <t>valorant-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="U85" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V85" s="24" t="n"/>
+      <c r="W85" s="26" t="n"/>
+      <c r="X85" s="26" t="n"/>
+      <c r="Y85" s="25" t="n"/>
+      <c r="Z85" s="26" t="n"/>
+      <c r="AA85" s="28" t="n"/>
+      <c r="AB85" s="28" t="n"/>
+      <c r="AC85" s="30" t="n"/>
+      <c r="AD85" s="24" t="n"/>
+      <c r="AE85" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=aec-valorant-kcg-aar-2026-07-23).</t>
+        </is>
+      </c>
+      <c r="AF85" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG85" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH85" s="24" t="n"/>
+      <c r="AI85" s="31" t="n"/>
+      <c r="AJ85" s="31" t="n"/>
+      <c r="AK85" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL85" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM85" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN85" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO85" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_LARGE_DISAGREEMENT_REVIEW</t>
+        </is>
+      </c>
+      <c r="AP85" s="24" t="inlineStr">
+        <is>
+          <t>ALTERNATE aTTaX Ruby</t>
+        </is>
+      </c>
+      <c r="AQ85" s="24" t="inlineStr">
+        <is>
+          <t>ALTERNATE aTTaX Ruby</t>
+        </is>
+      </c>
+      <c r="AR85" s="24" t="inlineStr">
+        <is>
+          <t>ALTERNATE aTTaX Ruby</t>
+        </is>
+      </c>
+      <c r="AS85" s="24" t="inlineStr">
+        <is>
+          <t>Karmine Corp GC</t>
+        </is>
+      </c>
+      <c r="AT85" s="24" t="inlineStr">
+        <is>
+          <t>Karmine Corp GC</t>
+        </is>
+      </c>
+      <c r="AU85" s="24" t="inlineStr">
+        <is>
+          <t>Karmine Corp GC</t>
+        </is>
+      </c>
+      <c r="AV85" s="24" t="n"/>
+      <c r="AW85" s="24" t="n"/>
+      <c r="AX85" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY85" s="24" t="n"/>
+      <c r="AZ85" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA85" s="24" t="inlineStr">
+        <is>
+          <t>df5a226c64918a54c70b8af3e0cd4abb6c4f42b67acb5547da319458502b0ed4</t>
+        </is>
+      </c>
+      <c r="BB85" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC85" s="24" t="inlineStr">
+        <is>
+          <t>valorant-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BD85" s="24" t="inlineStr">
+        <is>
+          <t>df5a226c64918a54c70b8af3e0cd4abb6c4f42b67acb5547da319458502b0ed4</t>
+        </is>
+      </c>
+      <c r="BE85" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF85" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG85" s="24" t="inlineStr">
+        <is>
+          <t>valorant-tiered-elo-v3</t>
+        </is>
+      </c>
+      <c r="BH85" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-23T16:36:43.922293Z</t>
+        </is>
+      </c>
+      <c r="BI85" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ85" s="25" t="n"/>
+      <c r="BK85" s="26" t="n">
+        <v>-163</v>
+      </c>
+      <c r="BL85" s="27" t="n">
+        <v>1.613497</v>
+      </c>
+      <c r="BM85" s="28" t="n">
+        <v>0.619772</v>
+      </c>
+      <c r="BN85" s="28" t="n"/>
+      <c r="BO85" s="28" t="n"/>
+      <c r="BP85" s="25" t="n"/>
+      <c r="BQ85" s="27" t="n"/>
+      <c r="BR85" s="28" t="n"/>
+      <c r="BS85" s="28" t="n"/>
+      <c r="BT85" s="28" t="n"/>
+      <c r="BU85" s="25" t="n"/>
+      <c r="BV85" s="29" t="n"/>
+      <c r="BW85" s="24" t="n"/>
+      <c r="BX85" s="30" t="n"/>
+      <c r="BY85" s="27" t="n"/>
+      <c r="BZ85" s="24" t="n"/>
+      <c r="CA85" s="31" t="n"/>
+      <c r="CB85" s="24" t="n"/>
+      <c r="CC85" s="24" t="n"/>
+      <c r="CD85" s="24" t="n"/>
+      <c r="CE85" s="24" t="n"/>
+      <c r="CF85" s="24" t="n"/>
+      <c r="CG85" s="24" t="n"/>
+      <c r="CH85" s="24" t="n"/>
+      <c r="CI85" s="24" t="n"/>
+      <c r="CJ85" s="24" t="n"/>
+      <c r="CK85" s="24" t="n"/>
+      <c r="CL85" s="24" t="n"/>
+      <c r="CM85" s="24" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>